<commit_message>
feat: Atenza App v5.0 - Quotations conversion, Job Orders & Live Workshop Tracker, Role Permissions Matrix, Smart Navigation, and updated README
</commit_message>
<xml_diff>
--- a/Salaries.xlsx
+++ b/Salaries.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\OneDrive\Desktop\Workshop_manger_v2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\OneDrive\Desktop\Month_4\Salaries\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{340B5D6D-2E43-4CBA-BE53-D0EF2053118B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65F087F9-ABAE-4CE9-8160-112C357A89E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="19125" windowHeight="15585" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="مخطط1" sheetId="2" r:id="rId1"/>
@@ -44,6 +44,7 @@
     <author>tc={75608FF2-3075-452B-AE83-321CC302886C}</author>
     <author>tc={59E96417-C488-414C-B333-5E8432E1542E}</author>
     <author>tc={7D5C8E9C-844A-45F2-AEC7-F3760C8C3FDA}</author>
+    <author>tc={5F4C2469-C911-407B-AC23-486A3D18408E}</author>
     <author>tc={1F91E0B7-1447-4AF5-8C4B-8A571C44245A}</author>
   </authors>
   <commentList>
@@ -88,7 +89,15 @@
 </t>
       </text>
     </comment>
-    <comment ref="B36" authorId="5" shapeId="0" xr:uid="{1F91E0B7-1447-4AF5-8C4B-8A571C44245A}">
+    <comment ref="F22" authorId="5" shapeId="0" xr:uid="{5F4C2469-C911-407B-AC23-486A3D18408E}">
+      <text>
+        <t>[تعليق مترابط]
+الإصدار المثبت لديك من Excel يسمح لك بقراءة هذا التعليق المترابط؛ ومع ذلك، ستتم إزالة أي تعديلات أُجريت عليه إذا تم فتح الملف في إصدار أحدث من Excel. تعرّف على المزيد على:https://go.microsoft.com/fwlink/?linkid=870924
+التعليق:
+    حسم مخالفة مرورية 225</t>
+      </text>
+    </comment>
+    <comment ref="B36" authorId="6" shapeId="0" xr:uid="{1F91E0B7-1447-4AF5-8C4B-8A571C44245A}">
       <text>
         <t>[تعليق مترابط]
 الإصدار المثبت لديك من Excel يسمح لك بقراءة هذا التعليق المترابط؛ ومع ذلك، ستتم إزالة أي تعديلات أُجريت عليه إذا تم فتح الملف في إصدار أحدث من Excel. تعرّف على المزيد على:https://go.microsoft.com/fwlink/?linkid=870924
@@ -124,6 +133,9 @@
     <t xml:space="preserve">رواتب </t>
   </si>
   <si>
+    <t>الراتب الاساسي</t>
+  </si>
+  <si>
     <t>ايداع مؤسسة</t>
   </si>
   <si>
@@ -131,6 +143,9 @@
   </si>
   <si>
     <t>اجمالي السحبيات</t>
+  </si>
+  <si>
+    <t>المتبقي من راتب اساسي</t>
   </si>
   <si>
     <t xml:space="preserve">المتبقي  الصافي </t>
@@ -197,12 +212,6 @@
   </si>
   <si>
     <t>samer-wahid</t>
-  </si>
-  <si>
-    <t>الراتب الأساسي</t>
-  </si>
-  <si>
-    <t>الراتب المتبقي</t>
   </si>
   <si>
     <t>yaqoob</t>
@@ -539,7 +548,6 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="16" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="16" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -603,9 +611,6 @@
     <xf numFmtId="0" fontId="9" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -616,21 +621,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="عادي" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="50">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="47">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -657,34 +658,6 @@
       </fill>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
@@ -1235,6 +1208,9 @@
                   <c:pt idx="15">
                     <c:v>500</c:v>
                   </c:pt>
+                  <c:pt idx="22">
+                    <c:v>400</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="7">
@@ -1252,6 +1228,12 @@
                   <c:pt idx="15">
                     <c:v>400</c:v>
                   </c:pt>
+                  <c:pt idx="20">
+                    <c:v>200</c:v>
+                  </c:pt>
+                  <c:pt idx="22">
+                    <c:v>500</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="0">
@@ -1290,6 +1272,21 @@
                   <c:pt idx="17">
                     <c:v>70</c:v>
                   </c:pt>
+                  <c:pt idx="19">
+                    <c:v>250</c:v>
+                  </c:pt>
+                  <c:pt idx="20">
+                    <c:v>240</c:v>
+                  </c:pt>
+                  <c:pt idx="21">
+                    <c:v>50</c:v>
+                  </c:pt>
+                  <c:pt idx="22">
+                    <c:v>215</c:v>
+                  </c:pt>
+                  <c:pt idx="24">
+                    <c:v>10</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="8">
@@ -1298,6 +1295,9 @@
                   <c:pt idx="15">
                     <c:v>700</c:v>
                   </c:pt>
+                  <c:pt idx="22">
+                    <c:v>500</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="0">
@@ -1336,6 +1336,18 @@
                   <c:pt idx="18">
                     <c:v>100</c:v>
                   </c:pt>
+                  <c:pt idx="19">
+                    <c:v>150</c:v>
+                  </c:pt>
+                  <c:pt idx="21">
+                    <c:v>50</c:v>
+                  </c:pt>
+                  <c:pt idx="22">
+                    <c:v>300</c:v>
+                  </c:pt>
+                  <c:pt idx="24">
+                    <c:v>100</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="0">
@@ -1374,6 +1386,15 @@
                   <c:pt idx="18">
                     <c:v>50</c:v>
                   </c:pt>
+                  <c:pt idx="20">
+                    <c:v>110</c:v>
+                  </c:pt>
+                  <c:pt idx="21">
+                    <c:v>60</c:v>
+                  </c:pt>
+                  <c:pt idx="22">
+                    <c:v>200</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="5">
@@ -1396,6 +1417,12 @@
                   </c:pt>
                   <c:pt idx="18">
                     <c:v>200</c:v>
+                  </c:pt>
+                  <c:pt idx="22">
+                    <c:v>400</c:v>
+                  </c:pt>
+                  <c:pt idx="24">
+                    <c:v>35</c:v>
                   </c:pt>
                 </c:lvl>
                 <c:lvl>
@@ -1657,6 +1684,9 @@
                   <c:pt idx="15">
                     <c:v>500</c:v>
                   </c:pt>
+                  <c:pt idx="22">
+                    <c:v>400</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="7">
@@ -1674,6 +1704,12 @@
                   <c:pt idx="15">
                     <c:v>400</c:v>
                   </c:pt>
+                  <c:pt idx="20">
+                    <c:v>200</c:v>
+                  </c:pt>
+                  <c:pt idx="22">
+                    <c:v>500</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="0">
@@ -1712,6 +1748,21 @@
                   <c:pt idx="17">
                     <c:v>70</c:v>
                   </c:pt>
+                  <c:pt idx="19">
+                    <c:v>250</c:v>
+                  </c:pt>
+                  <c:pt idx="20">
+                    <c:v>240</c:v>
+                  </c:pt>
+                  <c:pt idx="21">
+                    <c:v>50</c:v>
+                  </c:pt>
+                  <c:pt idx="22">
+                    <c:v>215</c:v>
+                  </c:pt>
+                  <c:pt idx="24">
+                    <c:v>10</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="8">
@@ -1720,6 +1771,9 @@
                   <c:pt idx="15">
                     <c:v>700</c:v>
                   </c:pt>
+                  <c:pt idx="22">
+                    <c:v>500</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="0">
@@ -1758,6 +1812,18 @@
                   <c:pt idx="18">
                     <c:v>100</c:v>
                   </c:pt>
+                  <c:pt idx="19">
+                    <c:v>150</c:v>
+                  </c:pt>
+                  <c:pt idx="21">
+                    <c:v>50</c:v>
+                  </c:pt>
+                  <c:pt idx="22">
+                    <c:v>300</c:v>
+                  </c:pt>
+                  <c:pt idx="24">
+                    <c:v>100</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="0">
@@ -1796,6 +1862,15 @@
                   <c:pt idx="18">
                     <c:v>50</c:v>
                   </c:pt>
+                  <c:pt idx="20">
+                    <c:v>110</c:v>
+                  </c:pt>
+                  <c:pt idx="21">
+                    <c:v>60</c:v>
+                  </c:pt>
+                  <c:pt idx="22">
+                    <c:v>200</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="5">
@@ -1818,6 +1893,12 @@
                   </c:pt>
                   <c:pt idx="18">
                     <c:v>200</c:v>
+                  </c:pt>
+                  <c:pt idx="22">
+                    <c:v>400</c:v>
+                  </c:pt>
+                  <c:pt idx="24">
+                    <c:v>35</c:v>
                   </c:pt>
                 </c:lvl>
                 <c:lvl>
@@ -1926,6 +2007,9 @@
                 </c:pt>
                 <c:pt idx="15">
                   <c:v>500</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>200</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2067,6 +2151,9 @@
                   <c:pt idx="15">
                     <c:v>500</c:v>
                   </c:pt>
+                  <c:pt idx="22">
+                    <c:v>400</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="7">
@@ -2084,6 +2171,12 @@
                   <c:pt idx="15">
                     <c:v>400</c:v>
                   </c:pt>
+                  <c:pt idx="20">
+                    <c:v>200</c:v>
+                  </c:pt>
+                  <c:pt idx="22">
+                    <c:v>500</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="0">
@@ -2122,6 +2215,21 @@
                   <c:pt idx="17">
                     <c:v>70</c:v>
                   </c:pt>
+                  <c:pt idx="19">
+                    <c:v>250</c:v>
+                  </c:pt>
+                  <c:pt idx="20">
+                    <c:v>240</c:v>
+                  </c:pt>
+                  <c:pt idx="21">
+                    <c:v>50</c:v>
+                  </c:pt>
+                  <c:pt idx="22">
+                    <c:v>215</c:v>
+                  </c:pt>
+                  <c:pt idx="24">
+                    <c:v>10</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="8">
@@ -2130,6 +2238,9 @@
                   <c:pt idx="15">
                     <c:v>700</c:v>
                   </c:pt>
+                  <c:pt idx="22">
+                    <c:v>500</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="0">
@@ -2168,6 +2279,18 @@
                   <c:pt idx="18">
                     <c:v>100</c:v>
                   </c:pt>
+                  <c:pt idx="19">
+                    <c:v>150</c:v>
+                  </c:pt>
+                  <c:pt idx="21">
+                    <c:v>50</c:v>
+                  </c:pt>
+                  <c:pt idx="22">
+                    <c:v>300</c:v>
+                  </c:pt>
+                  <c:pt idx="24">
+                    <c:v>100</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="0">
@@ -2206,6 +2329,15 @@
                   <c:pt idx="18">
                     <c:v>50</c:v>
                   </c:pt>
+                  <c:pt idx="20">
+                    <c:v>110</c:v>
+                  </c:pt>
+                  <c:pt idx="21">
+                    <c:v>60</c:v>
+                  </c:pt>
+                  <c:pt idx="22">
+                    <c:v>200</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="5">
@@ -2228,6 +2360,12 @@
                   </c:pt>
                   <c:pt idx="18">
                     <c:v>200</c:v>
+                  </c:pt>
+                  <c:pt idx="22">
+                    <c:v>400</c:v>
+                  </c:pt>
+                  <c:pt idx="24">
+                    <c:v>35</c:v>
                   </c:pt>
                 </c:lvl>
                 <c:lvl>
@@ -2489,6 +2627,9 @@
                   <c:pt idx="15">
                     <c:v>500</c:v>
                   </c:pt>
+                  <c:pt idx="22">
+                    <c:v>400</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="7">
@@ -2506,6 +2647,12 @@
                   <c:pt idx="15">
                     <c:v>400</c:v>
                   </c:pt>
+                  <c:pt idx="20">
+                    <c:v>200</c:v>
+                  </c:pt>
+                  <c:pt idx="22">
+                    <c:v>500</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="0">
@@ -2544,6 +2691,21 @@
                   <c:pt idx="17">
                     <c:v>70</c:v>
                   </c:pt>
+                  <c:pt idx="19">
+                    <c:v>250</c:v>
+                  </c:pt>
+                  <c:pt idx="20">
+                    <c:v>240</c:v>
+                  </c:pt>
+                  <c:pt idx="21">
+                    <c:v>50</c:v>
+                  </c:pt>
+                  <c:pt idx="22">
+                    <c:v>215</c:v>
+                  </c:pt>
+                  <c:pt idx="24">
+                    <c:v>10</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="8">
@@ -2552,6 +2714,9 @@
                   <c:pt idx="15">
                     <c:v>700</c:v>
                   </c:pt>
+                  <c:pt idx="22">
+                    <c:v>500</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="0">
@@ -2590,6 +2755,18 @@
                   <c:pt idx="18">
                     <c:v>100</c:v>
                   </c:pt>
+                  <c:pt idx="19">
+                    <c:v>150</c:v>
+                  </c:pt>
+                  <c:pt idx="21">
+                    <c:v>50</c:v>
+                  </c:pt>
+                  <c:pt idx="22">
+                    <c:v>300</c:v>
+                  </c:pt>
+                  <c:pt idx="24">
+                    <c:v>100</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="0">
@@ -2628,6 +2805,15 @@
                   <c:pt idx="18">
                     <c:v>50</c:v>
                   </c:pt>
+                  <c:pt idx="20">
+                    <c:v>110</c:v>
+                  </c:pt>
+                  <c:pt idx="21">
+                    <c:v>60</c:v>
+                  </c:pt>
+                  <c:pt idx="22">
+                    <c:v>200</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="5">
@@ -2650,6 +2836,12 @@
                   </c:pt>
                   <c:pt idx="18">
                     <c:v>200</c:v>
+                  </c:pt>
+                  <c:pt idx="22">
+                    <c:v>400</c:v>
+                  </c:pt>
+                  <c:pt idx="24">
+                    <c:v>35</c:v>
                   </c:pt>
                 </c:lvl>
                 <c:lvl>
@@ -2902,6 +3094,9 @@
                   <c:pt idx="15">
                     <c:v>500</c:v>
                   </c:pt>
+                  <c:pt idx="22">
+                    <c:v>400</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="7">
@@ -2919,6 +3114,12 @@
                   <c:pt idx="15">
                     <c:v>400</c:v>
                   </c:pt>
+                  <c:pt idx="20">
+                    <c:v>200</c:v>
+                  </c:pt>
+                  <c:pt idx="22">
+                    <c:v>500</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="0">
@@ -2957,6 +3158,21 @@
                   <c:pt idx="17">
                     <c:v>70</c:v>
                   </c:pt>
+                  <c:pt idx="19">
+                    <c:v>250</c:v>
+                  </c:pt>
+                  <c:pt idx="20">
+                    <c:v>240</c:v>
+                  </c:pt>
+                  <c:pt idx="21">
+                    <c:v>50</c:v>
+                  </c:pt>
+                  <c:pt idx="22">
+                    <c:v>215</c:v>
+                  </c:pt>
+                  <c:pt idx="24">
+                    <c:v>10</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="8">
@@ -2965,6 +3181,9 @@
                   <c:pt idx="15">
                     <c:v>700</c:v>
                   </c:pt>
+                  <c:pt idx="22">
+                    <c:v>500</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="0">
@@ -3003,6 +3222,18 @@
                   <c:pt idx="18">
                     <c:v>100</c:v>
                   </c:pt>
+                  <c:pt idx="19">
+                    <c:v>150</c:v>
+                  </c:pt>
+                  <c:pt idx="21">
+                    <c:v>50</c:v>
+                  </c:pt>
+                  <c:pt idx="22">
+                    <c:v>300</c:v>
+                  </c:pt>
+                  <c:pt idx="24">
+                    <c:v>100</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="0">
@@ -3041,6 +3272,15 @@
                   <c:pt idx="18">
                     <c:v>50</c:v>
                   </c:pt>
+                  <c:pt idx="20">
+                    <c:v>110</c:v>
+                  </c:pt>
+                  <c:pt idx="21">
+                    <c:v>60</c:v>
+                  </c:pt>
+                  <c:pt idx="22">
+                    <c:v>200</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="5">
@@ -3063,6 +3303,12 @@
                   </c:pt>
                   <c:pt idx="18">
                     <c:v>200</c:v>
+                  </c:pt>
+                  <c:pt idx="22">
+                    <c:v>400</c:v>
+                  </c:pt>
+                  <c:pt idx="24">
+                    <c:v>35</c:v>
                   </c:pt>
                 </c:lvl>
                 <c:lvl>
@@ -3309,6 +3555,9 @@
                   <c:pt idx="15">
                     <c:v>500</c:v>
                   </c:pt>
+                  <c:pt idx="22">
+                    <c:v>400</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="7">
@@ -3326,6 +3575,12 @@
                   <c:pt idx="15">
                     <c:v>400</c:v>
                   </c:pt>
+                  <c:pt idx="20">
+                    <c:v>200</c:v>
+                  </c:pt>
+                  <c:pt idx="22">
+                    <c:v>500</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="0">
@@ -3364,6 +3619,21 @@
                   <c:pt idx="17">
                     <c:v>70</c:v>
                   </c:pt>
+                  <c:pt idx="19">
+                    <c:v>250</c:v>
+                  </c:pt>
+                  <c:pt idx="20">
+                    <c:v>240</c:v>
+                  </c:pt>
+                  <c:pt idx="21">
+                    <c:v>50</c:v>
+                  </c:pt>
+                  <c:pt idx="22">
+                    <c:v>215</c:v>
+                  </c:pt>
+                  <c:pt idx="24">
+                    <c:v>10</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="8">
@@ -3372,6 +3642,9 @@
                   <c:pt idx="15">
                     <c:v>700</c:v>
                   </c:pt>
+                  <c:pt idx="22">
+                    <c:v>500</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="0">
@@ -3410,6 +3683,18 @@
                   <c:pt idx="18">
                     <c:v>100</c:v>
                   </c:pt>
+                  <c:pt idx="19">
+                    <c:v>150</c:v>
+                  </c:pt>
+                  <c:pt idx="21">
+                    <c:v>50</c:v>
+                  </c:pt>
+                  <c:pt idx="22">
+                    <c:v>300</c:v>
+                  </c:pt>
+                  <c:pt idx="24">
+                    <c:v>100</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="0">
@@ -3448,6 +3733,15 @@
                   <c:pt idx="18">
                     <c:v>50</c:v>
                   </c:pt>
+                  <c:pt idx="20">
+                    <c:v>110</c:v>
+                  </c:pt>
+                  <c:pt idx="21">
+                    <c:v>60</c:v>
+                  </c:pt>
+                  <c:pt idx="22">
+                    <c:v>200</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="5">
@@ -3470,6 +3764,12 @@
                   </c:pt>
                   <c:pt idx="18">
                     <c:v>200</c:v>
+                  </c:pt>
+                  <c:pt idx="22">
+                    <c:v>400</c:v>
+                  </c:pt>
+                  <c:pt idx="24">
+                    <c:v>35</c:v>
                   </c:pt>
                 </c:lvl>
                 <c:lvl>
@@ -3587,6 +3887,12 @@
                 </c:pt>
                 <c:pt idx="15">
                   <c:v>700</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>400</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3730,6 +4036,9 @@
                   <c:pt idx="15">
                     <c:v>500</c:v>
                   </c:pt>
+                  <c:pt idx="22">
+                    <c:v>400</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="7">
@@ -3747,6 +4056,12 @@
                   <c:pt idx="15">
                     <c:v>400</c:v>
                   </c:pt>
+                  <c:pt idx="20">
+                    <c:v>200</c:v>
+                  </c:pt>
+                  <c:pt idx="22">
+                    <c:v>500</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="0">
@@ -3785,6 +4100,21 @@
                   <c:pt idx="17">
                     <c:v>70</c:v>
                   </c:pt>
+                  <c:pt idx="19">
+                    <c:v>250</c:v>
+                  </c:pt>
+                  <c:pt idx="20">
+                    <c:v>240</c:v>
+                  </c:pt>
+                  <c:pt idx="21">
+                    <c:v>50</c:v>
+                  </c:pt>
+                  <c:pt idx="22">
+                    <c:v>215</c:v>
+                  </c:pt>
+                  <c:pt idx="24">
+                    <c:v>10</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="8">
@@ -3793,6 +4123,9 @@
                   <c:pt idx="15">
                     <c:v>700</c:v>
                   </c:pt>
+                  <c:pt idx="22">
+                    <c:v>500</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="0">
@@ -3831,6 +4164,18 @@
                   <c:pt idx="18">
                     <c:v>100</c:v>
                   </c:pt>
+                  <c:pt idx="19">
+                    <c:v>150</c:v>
+                  </c:pt>
+                  <c:pt idx="21">
+                    <c:v>50</c:v>
+                  </c:pt>
+                  <c:pt idx="22">
+                    <c:v>300</c:v>
+                  </c:pt>
+                  <c:pt idx="24">
+                    <c:v>100</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="0">
@@ -3869,6 +4214,15 @@
                   <c:pt idx="18">
                     <c:v>50</c:v>
                   </c:pt>
+                  <c:pt idx="20">
+                    <c:v>110</c:v>
+                  </c:pt>
+                  <c:pt idx="21">
+                    <c:v>60</c:v>
+                  </c:pt>
+                  <c:pt idx="22">
+                    <c:v>200</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="5">
@@ -3891,6 +4245,12 @@
                   </c:pt>
                   <c:pt idx="18">
                     <c:v>200</c:v>
+                  </c:pt>
+                  <c:pt idx="22">
+                    <c:v>400</c:v>
+                  </c:pt>
+                  <c:pt idx="24">
+                    <c:v>35</c:v>
                   </c:pt>
                 </c:lvl>
                 <c:lvl>
@@ -4791,37 +5151,37 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Fut Abd" id="{2A37FB36-686A-4E2D-80DD-FF2A12DF4263}" userId="98ea0cd7aab4f1fb" providerId="Windows Live"/>
   <person displayName="A" id="{58B860D6-0B45-4D13-BFB1-FF47055B2BB5}" userId="S::dd52@QuadClouds.onmicrosoft.com::b7d8920b-3ce6-4d86-8b8e-8873cd508aed" providerId="AD"/>
 </personList>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{638CBA3A-5512-460D-B773-5DABB0E16099}" name="الجدول1" displayName="الجدول1" ref="A2:V32" headerRowCount="0" totalsRowShown="0" headerRowDxfId="49" dataDxfId="48">
-  <tableColumns count="22">
-    <tableColumn id="1" xr3:uid="{4833D918-3E57-44BD-915B-DD91303766ED}" name="عمود1" headerRowDxfId="47" dataDxfId="46"/>
-    <tableColumn id="2" xr3:uid="{7B3FF86C-C28D-42DF-BD01-A4FE73ACE494}" name="عمود2" headerRowDxfId="45" dataDxfId="44"/>
-    <tableColumn id="3" xr3:uid="{31480497-3B1A-4412-82FD-B7918C79C323}" name="عمود3" headerRowDxfId="43" dataDxfId="42"/>
-    <tableColumn id="4" xr3:uid="{6D31A300-17B9-4587-9917-D67D3A1FAA21}" name="عمود4" headerRowDxfId="41" dataDxfId="40"/>
-    <tableColumn id="5" xr3:uid="{6443B874-742F-4A1C-A578-E3765B833858}" name="عمود5" headerRowDxfId="39" dataDxfId="38"/>
-    <tableColumn id="6" xr3:uid="{E9F26C06-1DF6-40F3-9147-654335FD38CD}" name="عمود6" headerRowDxfId="37" dataDxfId="36"/>
-    <tableColumn id="7" xr3:uid="{270BCF83-53C5-4720-9A1E-9C65C6D866DD}" name="عمود7" headerRowDxfId="35" dataDxfId="34"/>
-    <tableColumn id="8" xr3:uid="{3222AD16-160E-41A8-B516-706882EAB89A}" name="عمود8" headerRowDxfId="33" dataDxfId="32"/>
-    <tableColumn id="9" xr3:uid="{AF448870-039E-41DC-9F7B-669D47F6ABF9}" name="عمود9" headerRowDxfId="31" dataDxfId="30">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{638CBA3A-5512-460D-B773-5DABB0E16099}" name="الجدول1" displayName="الجدول1" ref="A2:U32" headerRowCount="0" totalsRowShown="0" headerRowDxfId="46" dataDxfId="45">
+  <tableColumns count="21">
+    <tableColumn id="1" xr3:uid="{4833D918-3E57-44BD-915B-DD91303766ED}" name="عمود1" headerRowDxfId="44" dataDxfId="43"/>
+    <tableColumn id="2" xr3:uid="{7B3FF86C-C28D-42DF-BD01-A4FE73ACE494}" name="عمود2" headerRowDxfId="42" dataDxfId="41"/>
+    <tableColumn id="3" xr3:uid="{31480497-3B1A-4412-82FD-B7918C79C323}" name="عمود3" headerRowDxfId="40" dataDxfId="39"/>
+    <tableColumn id="4" xr3:uid="{6D31A300-17B9-4587-9917-D67D3A1FAA21}" name="عمود4" headerRowDxfId="38" dataDxfId="37"/>
+    <tableColumn id="5" xr3:uid="{6443B874-742F-4A1C-A578-E3765B833858}" name="عمود5" headerRowDxfId="36" dataDxfId="35"/>
+    <tableColumn id="6" xr3:uid="{E9F26C06-1DF6-40F3-9147-654335FD38CD}" name="عمود6" headerRowDxfId="34" dataDxfId="33"/>
+    <tableColumn id="7" xr3:uid="{270BCF83-53C5-4720-9A1E-9C65C6D866DD}" name="عمود7" headerRowDxfId="32" dataDxfId="31"/>
+    <tableColumn id="8" xr3:uid="{3222AD16-160E-41A8-B516-706882EAB89A}" name="عمود8" headerRowDxfId="30" dataDxfId="29"/>
+    <tableColumn id="9" xr3:uid="{AF448870-039E-41DC-9F7B-669D47F6ABF9}" name="عمود9" headerRowDxfId="28" dataDxfId="27">
       <calculatedColumnFormula>+A3</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{8343A785-FE37-4FCF-AE05-71F27707D011}" name="عمود10" headerRowDxfId="29" dataDxfId="28"/>
-    <tableColumn id="11" xr3:uid="{B108BFD9-645F-4989-8F2D-A6EBFBF1DEFA}" name="عمود11" headerRowDxfId="27" dataDxfId="26"/>
-    <tableColumn id="12" xr3:uid="{33650B15-51C4-49E2-8196-1B276C844F8B}" name="عمود12" headerRowDxfId="25" dataDxfId="24"/>
-    <tableColumn id="13" xr3:uid="{18EA44B3-E4E0-49F3-A69A-5EAA7AE41E30}" name="عمود13" headerRowDxfId="23" dataDxfId="22"/>
-    <tableColumn id="14" xr3:uid="{8D4F979F-C562-4AEF-BFCA-6E8EF825EB72}" name="عمود14" headerRowDxfId="21" dataDxfId="20"/>
-    <tableColumn id="15" xr3:uid="{EFB0E8DC-CFAC-4645-8F85-24AF63D1C63B}" name="عمود15" headerRowDxfId="19" dataDxfId="18"/>
-    <tableColumn id="16" xr3:uid="{9ECE0C0A-FF62-46E6-85E8-C3CB68176A84}" name="عمود16" headerRowDxfId="17" dataDxfId="16"/>
-    <tableColumn id="18" xr3:uid="{F5526E9F-AD15-43BA-951A-7976A86F572D}" name="عمود18" headerRowDxfId="15" dataDxfId="14"/>
-    <tableColumn id="19" xr3:uid="{3AF7B6A2-514F-4540-9C54-C99E65C6E6DB}" name="عمود19" headerRowDxfId="13" dataDxfId="12"/>
-    <tableColumn id="20" xr3:uid="{97E00850-7A44-4BE3-8DF5-CFA90C6230F4}" name="عمود20" headerRowDxfId="11" dataDxfId="10"/>
-    <tableColumn id="21" xr3:uid="{FD53C09D-44A2-4510-A96B-A701193735BC}" name="عمود21" headerRowDxfId="9" dataDxfId="8"/>
-    <tableColumn id="22" xr3:uid="{80DE3AFF-B7BA-4304-8494-11970CF29614}" name="عمود22" headerRowDxfId="7" dataDxfId="6"/>
-    <tableColumn id="17" xr3:uid="{59CD8AD4-6BBB-472E-B26E-3011EF1B4AFD}" name="عمود17" headerRowDxfId="5" dataDxfId="4"/>
+    <tableColumn id="10" xr3:uid="{8343A785-FE37-4FCF-AE05-71F27707D011}" name="عمود10" headerRowDxfId="26" dataDxfId="25"/>
+    <tableColumn id="11" xr3:uid="{B108BFD9-645F-4989-8F2D-A6EBFBF1DEFA}" name="عمود11" headerRowDxfId="24" dataDxfId="23"/>
+    <tableColumn id="12" xr3:uid="{33650B15-51C4-49E2-8196-1B276C844F8B}" name="عمود12" headerRowDxfId="22" dataDxfId="21"/>
+    <tableColumn id="13" xr3:uid="{18EA44B3-E4E0-49F3-A69A-5EAA7AE41E30}" name="عمود13" headerRowDxfId="20" dataDxfId="19"/>
+    <tableColumn id="14" xr3:uid="{8D4F979F-C562-4AEF-BFCA-6E8EF825EB72}" name="عمود14" headerRowDxfId="18" dataDxfId="17"/>
+    <tableColumn id="15" xr3:uid="{EFB0E8DC-CFAC-4645-8F85-24AF63D1C63B}" name="عمود15" headerRowDxfId="16" dataDxfId="15"/>
+    <tableColumn id="16" xr3:uid="{9ECE0C0A-FF62-46E6-85E8-C3CB68176A84}" name="عمود16" headerRowDxfId="14" dataDxfId="13"/>
+    <tableColumn id="18" xr3:uid="{F5526E9F-AD15-43BA-951A-7976A86F572D}" name="عمود18" headerRowDxfId="12" dataDxfId="11"/>
+    <tableColumn id="19" xr3:uid="{3AF7B6A2-514F-4540-9C54-C99E65C6E6DB}" name="عمود19" headerRowDxfId="10" dataDxfId="9"/>
+    <tableColumn id="20" xr3:uid="{97E00850-7A44-4BE3-8DF5-CFA90C6230F4}" name="عمود20" headerRowDxfId="8" dataDxfId="7"/>
+    <tableColumn id="21" xr3:uid="{FD53C09D-44A2-4510-A96B-A701193735BC}" name="عمود21" headerRowDxfId="6" dataDxfId="5"/>
+    <tableColumn id="17" xr3:uid="{59CD8AD4-6BBB-472E-B26E-3011EF1B4AFD}" name="عمود17" headerRowDxfId="4" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="1"/>
 </table>
@@ -5106,6 +5466,9 @@
     <text xml:space="preserve">رجيع طبة رديتر انوفا 80
 </text>
   </threadedComment>
+  <threadedComment ref="F22" dT="2026-04-23T07:05:17.30" personId="{2A37FB36-686A-4E2D-80DD-FF2A12DF4263}" id="{5F4C2469-C911-407B-AC23-486A3D18408E}">
+    <text>حسم مخالفة مرورية 225</text>
+  </threadedComment>
   <threadedComment ref="B36" dT="2026-02-03T08:35:19.42" personId="{58B860D6-0B45-4D13-BFB1-FF47055B2BB5}" id="{1F91E0B7-1447-4AF5-8C4B-8A571C44245A}">
     <text>استرجاع راتب كاش 115</text>
   </threadedComment>
@@ -5117,10 +5480,10 @@
   <sheetPr codeName="ورقة1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Z42"/>
+  <dimension ref="A1:Y42"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.375" customWidth="1"/>
+    <col min="1" max="1" width="15.625" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="13.875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9.25" customWidth="1"/>
@@ -5132,1214 +5495,1277 @@
     <col min="16" max="16" width="9" customWidth="1"/>
     <col min="17" max="17" width="11.25" customWidth="1"/>
     <col min="19" max="20" width="8.625" customWidth="1"/>
-    <col min="21" max="22" width="10.375" customWidth="1"/>
-    <col min="23" max="23" width="11.625" customWidth="1"/>
-    <col min="24" max="24" width="9.375" customWidth="1"/>
-    <col min="25" max="25" width="10.875" customWidth="1"/>
-    <col min="26" max="26" width="12.375" customWidth="1"/>
+    <col min="21" max="21" width="10.375" customWidth="1"/>
+    <col min="22" max="22" width="11.625" customWidth="1"/>
+    <col min="23" max="23" width="9.375" customWidth="1"/>
+    <col min="24" max="24" width="10.875" customWidth="1"/>
+    <col min="25" max="25" width="12.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="19" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1" s="38" t="s">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="C1" s="37" t="s">
+        <v>14</v>
       </c>
       <c r="D1" s="19" t="s">
-        <v>13</v>
-      </c>
-      <c r="E1" s="38" t="s">
-        <v>31</v>
-      </c>
-      <c r="F1" s="38" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="E1" s="37" t="s">
+        <v>33</v>
+      </c>
+      <c r="F1" s="37" t="s">
+        <v>16</v>
       </c>
       <c r="G1" s="17" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H1" s="17" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="I1" s="20" t="s">
         <v>0</v>
       </c>
       <c r="J1" s="17" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="K1" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="L1" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="N1" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="O1" s="31" t="s">
+        <v>24</v>
+      </c>
+      <c r="P1" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="L1" s="33" t="s">
+      <c r="Q1" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="R1" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="M1" s="17" t="s">
-        <v>17</v>
-      </c>
-      <c r="N1" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="O1" s="32" t="s">
-        <v>22</v>
-      </c>
-      <c r="P1" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="Q1" s="21" t="s">
-        <v>20</v>
-      </c>
-      <c r="R1" s="21" t="s">
-        <v>23</v>
-      </c>
       <c r="S1" s="21" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="T1" s="19" t="s">
-        <v>24</v>
-      </c>
-      <c r="U1" s="64"/>
-      <c r="V1" s="65" t="s">
+        <v>26</v>
+      </c>
+      <c r="U1" s="63" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A2" s="23">
         <v>45748</v>
       </c>
       <c r="B2" s="1"/>
-      <c r="C2" s="59">
+      <c r="C2" s="58">
         <v>50</v>
       </c>
       <c r="D2" s="1">
         <v>250</v>
       </c>
-      <c r="E2" s="59"/>
-      <c r="F2" s="66">
+      <c r="E2" s="58"/>
+      <c r="F2" s="64">
         <v>1903.74</v>
       </c>
-      <c r="G2" s="47"/>
-      <c r="H2" s="47"/>
+      <c r="G2" s="46"/>
+      <c r="H2" s="46"/>
       <c r="I2" s="23">
         <f t="shared" ref="I2:I31" si="0">+A2</f>
         <v>45748</v>
       </c>
-      <c r="J2" s="49">
+      <c r="J2" s="48">
         <v>30</v>
       </c>
-      <c r="K2" s="66"/>
-      <c r="L2" s="66"/>
-      <c r="M2" s="66"/>
-      <c r="N2" s="47"/>
-      <c r="O2" s="66"/>
-      <c r="P2" s="56"/>
-      <c r="Q2" s="56"/>
-      <c r="R2" s="66"/>
-      <c r="S2" s="56"/>
+      <c r="K2" s="64"/>
+      <c r="L2" s="64"/>
+      <c r="M2" s="64"/>
+      <c r="N2" s="46"/>
+      <c r="O2" s="64"/>
+      <c r="P2" s="55"/>
+      <c r="Q2" s="55"/>
+      <c r="R2" s="64"/>
+      <c r="S2" s="55"/>
       <c r="T2" s="1"/>
-      <c r="V2" s="59"/>
+      <c r="U2" s="58"/>
     </row>
-    <row r="3" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="23">
         <v>45749</v>
       </c>
       <c r="B3" s="1"/>
-      <c r="C3" s="62"/>
+      <c r="C3" s="61"/>
       <c r="D3" s="1">
         <v>200</v>
       </c>
-      <c r="E3" s="59"/>
-      <c r="F3" s="59"/>
-      <c r="G3" s="47"/>
-      <c r="H3" s="47"/>
+      <c r="E3" s="58"/>
+      <c r="F3" s="58"/>
+      <c r="G3" s="46"/>
+      <c r="H3" s="46"/>
       <c r="I3" s="23">
         <f t="shared" si="0"/>
         <v>45749</v>
       </c>
-      <c r="J3" s="49"/>
-      <c r="K3" s="47"/>
-      <c r="L3" s="66"/>
-      <c r="M3" s="47"/>
-      <c r="N3" s="47"/>
-      <c r="O3" s="66"/>
-      <c r="P3" s="56"/>
-      <c r="Q3" s="56"/>
-      <c r="R3" s="56"/>
-      <c r="S3" s="56"/>
+      <c r="J3" s="48"/>
+      <c r="K3" s="46"/>
+      <c r="L3" s="64"/>
+      <c r="M3" s="46"/>
+      <c r="N3" s="46"/>
+      <c r="O3" s="64"/>
+      <c r="P3" s="55"/>
+      <c r="Q3" s="55"/>
+      <c r="R3" s="55"/>
+      <c r="S3" s="55"/>
       <c r="T3" s="1"/>
-      <c r="V3" s="59"/>
+      <c r="U3" s="58"/>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A4" s="31">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A4" s="30">
         <v>45750</v>
       </c>
       <c r="B4" s="1"/>
-      <c r="C4" s="62"/>
+      <c r="C4" s="61"/>
       <c r="D4" s="1"/>
-      <c r="E4" s="59"/>
-      <c r="F4" s="59"/>
-      <c r="G4" s="47"/>
-      <c r="H4" s="47"/>
-      <c r="I4" s="31">
+      <c r="E4" s="58"/>
+      <c r="F4" s="58"/>
+      <c r="G4" s="46"/>
+      <c r="H4" s="46"/>
+      <c r="I4" s="30">
         <f t="shared" si="0"/>
         <v>45750</v>
       </c>
-      <c r="J4" s="49"/>
-      <c r="K4" s="47"/>
-      <c r="L4" s="47"/>
-      <c r="M4" s="47"/>
-      <c r="N4" s="47"/>
-      <c r="O4" s="48"/>
-      <c r="P4" s="56"/>
-      <c r="Q4" s="56"/>
-      <c r="R4" s="56"/>
-      <c r="S4" s="56"/>
+      <c r="J4" s="48"/>
+      <c r="K4" s="46"/>
+      <c r="L4" s="46"/>
+      <c r="M4" s="46"/>
+      <c r="N4" s="46"/>
+      <c r="O4" s="47"/>
+      <c r="P4" s="55"/>
+      <c r="Q4" s="55"/>
+      <c r="R4" s="55"/>
+      <c r="S4" s="55"/>
       <c r="T4" s="1"/>
-      <c r="V4" s="59"/>
+      <c r="U4" s="58"/>
     </row>
-    <row r="5" spans="1:22" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:21" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="23">
         <v>45751</v>
       </c>
       <c r="B5" s="1"/>
-      <c r="C5" s="62"/>
+      <c r="C5" s="61"/>
       <c r="D5" s="1"/>
-      <c r="E5" s="59"/>
-      <c r="F5" s="59">
+      <c r="E5" s="58"/>
+      <c r="F5" s="58">
         <f>1900+1100</f>
         <v>3000</v>
       </c>
-      <c r="G5" s="66"/>
-      <c r="H5" s="47"/>
+      <c r="G5" s="64"/>
+      <c r="H5" s="46"/>
       <c r="I5" s="23">
         <f t="shared" si="0"/>
         <v>45751</v>
       </c>
-      <c r="J5" s="49">
+      <c r="J5" s="48">
         <v>150</v>
       </c>
-      <c r="K5" s="47"/>
-      <c r="L5" s="47"/>
-      <c r="M5" s="47">
+      <c r="K5" s="46"/>
+      <c r="L5" s="46"/>
+      <c r="M5" s="46">
         <v>109.48</v>
       </c>
-      <c r="N5" s="47"/>
-      <c r="O5" s="48">
+      <c r="N5" s="46"/>
+      <c r="O5" s="47">
         <v>200</v>
       </c>
-      <c r="P5" s="56"/>
-      <c r="Q5" s="56"/>
-      <c r="R5" s="56">
+      <c r="P5" s="55"/>
+      <c r="Q5" s="55"/>
+      <c r="R5" s="55">
         <v>6.87</v>
       </c>
-      <c r="S5" s="56">
+      <c r="S5" s="55">
         <v>100</v>
       </c>
       <c r="T5" s="1"/>
-      <c r="V5" s="59"/>
+      <c r="U5" s="58"/>
     </row>
-    <row r="6" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="23">
         <v>45752</v>
       </c>
       <c r="B6" s="1"/>
-      <c r="C6" s="62"/>
+      <c r="C6" s="61"/>
       <c r="D6" s="1">
         <v>100</v>
       </c>
-      <c r="E6" s="59"/>
-      <c r="F6" s="59"/>
-      <c r="G6" s="47"/>
-      <c r="H6" s="47"/>
+      <c r="E6" s="58"/>
+      <c r="F6" s="58"/>
+      <c r="G6" s="46"/>
+      <c r="H6" s="46"/>
       <c r="I6" s="23">
         <f t="shared" si="0"/>
         <v>45752</v>
       </c>
-      <c r="J6" s="49"/>
-      <c r="K6" s="50"/>
-      <c r="L6" s="47"/>
-      <c r="M6" s="47"/>
-      <c r="N6" s="47"/>
-      <c r="O6" s="47"/>
-      <c r="P6" s="56"/>
-      <c r="Q6" s="56"/>
-      <c r="R6" s="57"/>
-      <c r="S6" s="56"/>
+      <c r="J6" s="48"/>
+      <c r="K6" s="49"/>
+      <c r="L6" s="46"/>
+      <c r="M6" s="46"/>
+      <c r="N6" s="46"/>
+      <c r="O6" s="46"/>
+      <c r="P6" s="55"/>
+      <c r="Q6" s="55"/>
+      <c r="R6" s="56"/>
+      <c r="S6" s="55"/>
       <c r="T6" s="1"/>
-      <c r="V6" s="59"/>
+      <c r="U6" s="58"/>
     </row>
-    <row r="7" spans="1:22" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:21" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="23">
         <v>45753</v>
       </c>
       <c r="B7" s="1">
         <v>375</v>
       </c>
-      <c r="C7" s="62">
+      <c r="C7" s="61">
         <v>750</v>
       </c>
       <c r="D7" s="1">
         <v>750</v>
       </c>
-      <c r="E7" s="59"/>
-      <c r="F7" s="59">
+      <c r="E7" s="58"/>
+      <c r="F7" s="58">
         <f>20+500</f>
         <v>520</v>
       </c>
-      <c r="G7" s="47"/>
-      <c r="H7" s="47">
+      <c r="G7" s="46"/>
+      <c r="H7" s="46">
         <v>750</v>
       </c>
       <c r="I7" s="23">
         <f t="shared" si="0"/>
         <v>45753</v>
       </c>
-      <c r="J7" s="49"/>
-      <c r="K7" s="66"/>
-      <c r="L7" s="47">
+      <c r="J7" s="48"/>
+      <c r="K7" s="64"/>
+      <c r="L7" s="46">
         <v>750</v>
       </c>
-      <c r="M7" s="47">
+      <c r="M7" s="46">
         <v>750</v>
       </c>
-      <c r="N7" s="47">
+      <c r="N7" s="46">
         <v>750</v>
       </c>
-      <c r="O7" s="47"/>
-      <c r="P7" s="66">
+      <c r="O7" s="46"/>
+      <c r="P7" s="64">
         <v>375</v>
       </c>
-      <c r="Q7" s="56">
+      <c r="Q7" s="55">
         <v>750</v>
       </c>
-      <c r="R7" s="56">
+      <c r="R7" s="55">
         <f>4+750</f>
         <v>754</v>
       </c>
-      <c r="S7" s="56"/>
+      <c r="S7" s="55"/>
       <c r="T7" s="1"/>
-      <c r="V7" s="59"/>
+      <c r="U7" s="58"/>
     </row>
-    <row r="8" spans="1:22" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:21" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="23">
         <v>45754</v>
       </c>
       <c r="B8" s="1">
         <v>375</v>
       </c>
-      <c r="C8" s="62">
+      <c r="C8" s="61">
         <v>1250</v>
       </c>
       <c r="D8" s="1">
         <v>500</v>
       </c>
-      <c r="E8" s="59"/>
-      <c r="F8" s="59">
+      <c r="E8" s="58"/>
+      <c r="F8" s="58">
         <v>1200</v>
       </c>
-      <c r="G8" s="47"/>
-      <c r="H8" s="47"/>
+      <c r="G8" s="46"/>
+      <c r="H8" s="46"/>
       <c r="I8" s="23">
         <f t="shared" si="0"/>
         <v>45754</v>
       </c>
-      <c r="J8" s="49"/>
-      <c r="K8" s="47"/>
-      <c r="L8" s="47"/>
-      <c r="M8" s="47"/>
-      <c r="N8" s="47">
+      <c r="J8" s="48"/>
+      <c r="K8" s="46"/>
+      <c r="L8" s="46"/>
+      <c r="M8" s="46"/>
+      <c r="N8" s="46">
         <v>1350</v>
       </c>
-      <c r="O8" s="47"/>
-      <c r="P8" s="56"/>
-      <c r="Q8" s="56"/>
-      <c r="R8" s="56"/>
-      <c r="S8" s="56"/>
+      <c r="O8" s="46"/>
+      <c r="P8" s="55"/>
+      <c r="Q8" s="55"/>
+      <c r="R8" s="55"/>
+      <c r="S8" s="55"/>
       <c r="T8" s="1"/>
-      <c r="V8" s="59"/>
+      <c r="U8" s="58"/>
     </row>
-    <row r="9" spans="1:22" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:21" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="23">
         <v>45755</v>
       </c>
       <c r="B9" s="1"/>
-      <c r="C9" s="62">
+      <c r="C9" s="61">
         <v>50</v>
       </c>
       <c r="D9" s="1">
         <v>100</v>
       </c>
-      <c r="E9" s="59"/>
-      <c r="F9" s="59">
+      <c r="E9" s="58"/>
+      <c r="F9" s="58">
         <v>100</v>
       </c>
-      <c r="G9" s="47">
+      <c r="G9" s="46">
         <v>100</v>
       </c>
-      <c r="H9" s="47"/>
+      <c r="H9" s="46"/>
       <c r="I9" s="23">
         <f t="shared" si="0"/>
         <v>45755</v>
       </c>
-      <c r="J9" s="49">
+      <c r="J9" s="48">
         <v>20</v>
       </c>
-      <c r="K9" s="47"/>
-      <c r="L9" s="47"/>
-      <c r="M9" s="47"/>
-      <c r="N9" s="47"/>
-      <c r="O9" s="47"/>
-      <c r="P9" s="56"/>
-      <c r="Q9" s="56"/>
-      <c r="R9" s="56"/>
-      <c r="S9" s="56"/>
+      <c r="K9" s="46"/>
+      <c r="L9" s="46"/>
+      <c r="M9" s="46"/>
+      <c r="N9" s="46"/>
+      <c r="O9" s="46"/>
+      <c r="P9" s="55"/>
+      <c r="Q9" s="55"/>
+      <c r="R9" s="55"/>
+      <c r="S9" s="55"/>
       <c r="T9" s="1"/>
-      <c r="V9" s="59"/>
+      <c r="U9" s="58"/>
     </row>
-    <row r="10" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:21" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="23">
         <v>45756</v>
       </c>
       <c r="B10" s="1">
         <v>385.71</v>
       </c>
-      <c r="C10" s="62">
+      <c r="C10" s="61">
         <v>335.71</v>
       </c>
       <c r="D10" s="1">
         <v>1685.71</v>
       </c>
-      <c r="E10" s="59">
+      <c r="E10" s="58">
         <v>285.70999999999998</v>
       </c>
-      <c r="F10" s="59">
+      <c r="F10" s="58">
         <f>250+50+35.71</f>
         <v>335.71</v>
       </c>
-      <c r="G10" s="47">
+      <c r="G10" s="46">
         <v>535.71</v>
       </c>
-      <c r="H10" s="47">
+      <c r="H10" s="46">
         <v>1635.71</v>
       </c>
       <c r="I10" s="23">
         <f t="shared" si="0"/>
         <v>45756</v>
       </c>
-      <c r="J10" s="49">
+      <c r="J10" s="48">
         <f>400+300+35.71</f>
         <v>735.71</v>
       </c>
-      <c r="K10" s="47">
+      <c r="K10" s="46">
         <v>1000</v>
       </c>
-      <c r="L10" s="47">
+      <c r="L10" s="46">
         <v>35.71</v>
       </c>
-      <c r="M10" s="47">
+      <c r="M10" s="46">
         <v>535.71</v>
       </c>
-      <c r="N10" s="47">
+      <c r="N10" s="46">
         <v>150</v>
       </c>
-      <c r="O10" s="47"/>
-      <c r="P10" s="56">
+      <c r="O10" s="46"/>
+      <c r="P10" s="55">
         <f>200+35.71</f>
         <v>235.71</v>
       </c>
-      <c r="Q10" s="56">
+      <c r="Q10" s="55">
         <v>35.71</v>
       </c>
-      <c r="R10" s="56">
+      <c r="R10" s="55">
         <f>385.71+5+80</f>
         <v>470.71</v>
       </c>
-      <c r="S10" s="56">
+      <c r="S10" s="55">
         <v>100</v>
       </c>
       <c r="T10" s="1">
         <v>1235.71</v>
       </c>
-      <c r="V10" s="59"/>
+      <c r="U10" s="58"/>
     </row>
-    <row r="11" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="31">
+    <row r="11" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="30">
         <v>45757</v>
       </c>
       <c r="B11" s="1"/>
-      <c r="C11" s="62"/>
+      <c r="C11" s="61"/>
       <c r="D11" s="1"/>
-      <c r="E11" s="59"/>
-      <c r="F11" s="59"/>
-      <c r="G11" s="47"/>
-      <c r="H11" s="47"/>
-      <c r="I11" s="31">
+      <c r="E11" s="58"/>
+      <c r="F11" s="58"/>
+      <c r="G11" s="46"/>
+      <c r="H11" s="46"/>
+      <c r="I11" s="30">
         <f t="shared" si="0"/>
         <v>45757</v>
       </c>
-      <c r="J11" s="49"/>
-      <c r="K11" s="47"/>
-      <c r="L11" s="47"/>
-      <c r="M11" s="47"/>
-      <c r="N11" s="47"/>
-      <c r="O11" s="47"/>
-      <c r="P11" s="56"/>
-      <c r="Q11" s="56"/>
-      <c r="R11" s="56"/>
-      <c r="S11" s="56"/>
+      <c r="J11" s="48"/>
+      <c r="K11" s="46"/>
+      <c r="L11" s="46"/>
+      <c r="M11" s="46"/>
+      <c r="N11" s="46"/>
+      <c r="O11" s="46"/>
+      <c r="P11" s="55"/>
+      <c r="Q11" s="55"/>
+      <c r="R11" s="55"/>
+      <c r="S11" s="55"/>
       <c r="T11" s="1"/>
-      <c r="V11" s="59"/>
+      <c r="U11" s="58"/>
     </row>
-    <row r="12" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="23">
         <v>45758</v>
       </c>
       <c r="B12" s="1"/>
-      <c r="C12" s="62">
+      <c r="C12" s="61">
         <v>50</v>
       </c>
       <c r="D12" s="1"/>
-      <c r="E12" s="59"/>
-      <c r="F12" s="66"/>
-      <c r="G12" s="47"/>
-      <c r="H12" s="47"/>
+      <c r="E12" s="58"/>
+      <c r="F12" s="64"/>
+      <c r="G12" s="46"/>
+      <c r="H12" s="46"/>
       <c r="I12" s="23">
         <f t="shared" si="0"/>
         <v>45758</v>
       </c>
-      <c r="J12" s="49"/>
-      <c r="K12" s="47"/>
-      <c r="L12" s="47"/>
-      <c r="M12" s="47"/>
-      <c r="N12" s="47"/>
-      <c r="O12" s="47"/>
-      <c r="P12" s="56"/>
-      <c r="Q12" s="56"/>
-      <c r="R12" s="57">
+      <c r="J12" s="48"/>
+      <c r="K12" s="46"/>
+      <c r="L12" s="46"/>
+      <c r="M12" s="46"/>
+      <c r="N12" s="46"/>
+      <c r="O12" s="46"/>
+      <c r="P12" s="55"/>
+      <c r="Q12" s="55"/>
+      <c r="R12" s="56">
         <v>300</v>
       </c>
-      <c r="S12" s="56"/>
+      <c r="S12" s="55"/>
       <c r="T12" s="1"/>
-      <c r="V12" s="59"/>
+      <c r="U12" s="58"/>
     </row>
-    <row r="13" spans="1:22" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:21" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="23">
         <v>45759</v>
       </c>
-      <c r="B13" s="66"/>
-      <c r="C13" s="62">
+      <c r="B13" s="64"/>
+      <c r="C13" s="61">
         <v>50</v>
       </c>
       <c r="D13" s="1"/>
-      <c r="E13" s="59"/>
-      <c r="F13" s="59">
+      <c r="E13" s="58"/>
+      <c r="F13" s="58">
         <v>50</v>
       </c>
-      <c r="G13" s="47"/>
-      <c r="H13" s="47"/>
+      <c r="G13" s="46"/>
+      <c r="H13" s="46"/>
       <c r="I13" s="23">
         <f t="shared" si="0"/>
         <v>45759</v>
       </c>
-      <c r="J13" s="49"/>
-      <c r="K13" s="66"/>
-      <c r="L13" s="47"/>
-      <c r="M13" s="51"/>
-      <c r="N13" s="47"/>
-      <c r="O13" s="47"/>
-      <c r="P13" s="56"/>
-      <c r="Q13" s="56"/>
-      <c r="R13" s="66"/>
-      <c r="S13" s="56"/>
+      <c r="J13" s="48"/>
+      <c r="K13" s="64"/>
+      <c r="L13" s="46"/>
+      <c r="M13" s="50"/>
+      <c r="N13" s="46"/>
+      <c r="O13" s="46"/>
+      <c r="P13" s="55"/>
+      <c r="Q13" s="55"/>
+      <c r="R13" s="64"/>
+      <c r="S13" s="55"/>
       <c r="T13" s="1"/>
-      <c r="V13" s="59"/>
+      <c r="U13" s="58"/>
     </row>
-    <row r="14" spans="1:22" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:21" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="23">
         <v>45760</v>
       </c>
       <c r="B14" s="1">
         <v>600</v>
       </c>
-      <c r="C14" s="62">
+      <c r="C14" s="61">
         <v>100</v>
       </c>
       <c r="D14" s="1">
         <v>100</v>
       </c>
-      <c r="E14" s="59"/>
-      <c r="F14" s="59">
+      <c r="E14" s="58"/>
+      <c r="F14" s="58">
         <v>50</v>
       </c>
-      <c r="G14" s="47">
+      <c r="G14" s="46">
         <v>150</v>
       </c>
-      <c r="H14" s="47"/>
+      <c r="H14" s="46"/>
       <c r="I14" s="23">
         <f t="shared" si="0"/>
         <v>45760</v>
       </c>
-      <c r="J14" s="49"/>
-      <c r="K14" s="47"/>
-      <c r="L14" s="47"/>
-      <c r="M14" s="47"/>
-      <c r="N14" s="47"/>
-      <c r="O14" s="47"/>
-      <c r="P14" s="56"/>
-      <c r="Q14" s="56"/>
-      <c r="R14" s="56"/>
-      <c r="S14" s="56"/>
+      <c r="J14" s="48"/>
+      <c r="K14" s="46"/>
+      <c r="L14" s="46"/>
+      <c r="M14" s="46"/>
+      <c r="N14" s="46"/>
+      <c r="O14" s="46"/>
+      <c r="P14" s="55"/>
+      <c r="Q14" s="55"/>
+      <c r="R14" s="55"/>
+      <c r="S14" s="55"/>
       <c r="T14" s="1"/>
-      <c r="V14" s="59"/>
+      <c r="U14" s="58"/>
     </row>
-    <row r="15" spans="1:22" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:21" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="23">
         <v>45761</v>
       </c>
       <c r="B15" s="1"/>
-      <c r="C15" s="62">
+      <c r="C15" s="61">
         <v>650</v>
       </c>
       <c r="D15" s="1">
         <v>132.26</v>
       </c>
-      <c r="E15" s="59"/>
-      <c r="F15" s="59">
+      <c r="E15" s="58"/>
+      <c r="F15" s="58">
         <v>700</v>
       </c>
-      <c r="G15" s="47">
+      <c r="G15" s="46">
         <v>650</v>
       </c>
-      <c r="H15" s="47"/>
+      <c r="H15" s="46"/>
       <c r="I15" s="23">
         <f t="shared" si="0"/>
         <v>45761</v>
       </c>
-      <c r="J15" s="49"/>
-      <c r="K15" s="47"/>
-      <c r="L15" s="47"/>
-      <c r="M15" s="47">
+      <c r="J15" s="48"/>
+      <c r="K15" s="46"/>
+      <c r="L15" s="46"/>
+      <c r="M15" s="46">
         <v>50</v>
       </c>
-      <c r="N15" s="47"/>
-      <c r="O15" s="47"/>
-      <c r="P15" s="56"/>
-      <c r="Q15" s="56"/>
-      <c r="R15" s="57"/>
-      <c r="S15" s="56"/>
+      <c r="N15" s="46"/>
+      <c r="O15" s="46"/>
+      <c r="P15" s="55"/>
+      <c r="Q15" s="55"/>
+      <c r="R15" s="56"/>
+      <c r="S15" s="55"/>
       <c r="T15" s="1"/>
-      <c r="V15" s="59"/>
+      <c r="U15" s="58"/>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A16" s="23">
         <v>45762</v>
       </c>
       <c r="B16" s="1">
         <v>106</v>
       </c>
-      <c r="C16" s="62"/>
+      <c r="C16" s="61"/>
       <c r="D16" s="1"/>
-      <c r="E16" s="59"/>
-      <c r="F16" s="59">
+      <c r="E16" s="58"/>
+      <c r="F16" s="58">
         <v>35</v>
       </c>
-      <c r="G16" s="47"/>
-      <c r="H16" s="47"/>
+      <c r="G16" s="46"/>
+      <c r="H16" s="46"/>
       <c r="I16" s="23">
         <f t="shared" si="0"/>
         <v>45762</v>
       </c>
-      <c r="J16" s="49"/>
-      <c r="K16" s="47"/>
-      <c r="L16" s="47"/>
-      <c r="M16" s="47"/>
-      <c r="N16" s="47"/>
-      <c r="O16" s="47"/>
-      <c r="P16" s="56">
+      <c r="J16" s="48"/>
+      <c r="K16" s="46"/>
+      <c r="L16" s="46"/>
+      <c r="M16" s="46"/>
+      <c r="N16" s="46"/>
+      <c r="O16" s="46"/>
+      <c r="P16" s="55">
         <v>20</v>
       </c>
-      <c r="Q16" s="56"/>
-      <c r="R16" s="56">
+      <c r="Q16" s="55"/>
+      <c r="R16" s="55">
         <v>18.399999999999999</v>
       </c>
-      <c r="S16" s="56"/>
+      <c r="S16" s="55"/>
       <c r="T16" s="1"/>
-      <c r="V16" s="59"/>
+      <c r="U16" s="58"/>
     </row>
-    <row r="17" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A17" s="23">
         <v>45763</v>
       </c>
       <c r="B17" s="1">
         <v>550</v>
       </c>
-      <c r="C17" s="62">
+      <c r="C17" s="61">
         <f>50+200</f>
         <v>250</v>
       </c>
       <c r="D17" s="1">
         <v>100</v>
       </c>
-      <c r="E17" s="59">
+      <c r="E17" s="58">
         <v>700</v>
       </c>
-      <c r="F17" s="59">
+      <c r="F17" s="58">
         <v>100</v>
       </c>
-      <c r="G17" s="47">
+      <c r="G17" s="46">
         <v>400</v>
       </c>
-      <c r="H17" s="47">
+      <c r="H17" s="46">
         <v>500</v>
       </c>
       <c r="I17" s="23">
         <f t="shared" si="0"/>
         <v>45763</v>
       </c>
-      <c r="J17" s="49">
+      <c r="J17" s="48">
         <v>100</v>
       </c>
-      <c r="K17" s="47">
+      <c r="K17" s="46">
         <v>500</v>
       </c>
-      <c r="L17" s="47">
+      <c r="L17" s="46">
         <v>200</v>
       </c>
-      <c r="M17" s="52">
+      <c r="M17" s="51">
         <v>700</v>
       </c>
-      <c r="N17" s="52">
+      <c r="N17" s="51">
         <v>250</v>
       </c>
-      <c r="O17" s="52"/>
-      <c r="P17" s="56">
+      <c r="O17" s="51"/>
+      <c r="P17" s="55">
         <v>250</v>
       </c>
-      <c r="Q17" s="56">
+      <c r="Q17" s="55">
         <v>200</v>
       </c>
-      <c r="R17" s="56">
+      <c r="R17" s="55">
         <f>1250+40+650</f>
         <v>1940</v>
       </c>
-      <c r="S17" s="56">
+      <c r="S17" s="55">
         <v>100</v>
       </c>
       <c r="T17" s="1"/>
-      <c r="V17" s="59">
+      <c r="U17" s="58">
         <v>300</v>
       </c>
     </row>
-    <row r="18" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="A18" s="31">
+    <row r="18" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A18" s="30">
         <v>45764</v>
       </c>
       <c r="B18" s="1"/>
-      <c r="C18" s="62"/>
+      <c r="C18" s="61"/>
       <c r="D18" s="1"/>
-      <c r="E18" s="59"/>
-      <c r="F18" s="59"/>
-      <c r="G18" s="47"/>
-      <c r="H18" s="47"/>
-      <c r="I18" s="31">
+      <c r="E18" s="58"/>
+      <c r="F18" s="58"/>
+      <c r="G18" s="46"/>
+      <c r="H18" s="46"/>
+      <c r="I18" s="30">
         <f t="shared" si="0"/>
         <v>45764</v>
       </c>
-      <c r="J18" s="49"/>
-      <c r="K18" s="47"/>
-      <c r="L18" s="47"/>
-      <c r="M18" s="47"/>
-      <c r="N18" s="47"/>
-      <c r="O18" s="47"/>
-      <c r="P18" s="56"/>
-      <c r="Q18" s="56"/>
-      <c r="R18" s="56"/>
-      <c r="S18" s="56"/>
+      <c r="J18" s="48"/>
+      <c r="K18" s="46"/>
+      <c r="L18" s="46"/>
+      <c r="M18" s="46"/>
+      <c r="N18" s="46"/>
+      <c r="O18" s="46"/>
+      <c r="P18" s="55"/>
+      <c r="Q18" s="55"/>
+      <c r="R18" s="55"/>
+      <c r="S18" s="55"/>
       <c r="T18" s="1"/>
-      <c r="V18" s="59"/>
+      <c r="U18" s="58"/>
     </row>
-    <row r="19" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A19" s="23">
         <v>45765</v>
       </c>
       <c r="B19" s="1"/>
-      <c r="C19" s="62">
+      <c r="C19" s="61">
         <v>30</v>
       </c>
       <c r="D19" s="1">
         <f>70+56</f>
         <v>126</v>
       </c>
-      <c r="E19" s="59"/>
-      <c r="F19" s="59">
+      <c r="E19" s="58"/>
+      <c r="F19" s="58">
         <f>50+20</f>
         <v>70</v>
       </c>
-      <c r="G19" s="47"/>
-      <c r="H19" s="47"/>
+      <c r="G19" s="46"/>
+      <c r="H19" s="46"/>
       <c r="I19" s="23">
         <f t="shared" si="0"/>
         <v>45765</v>
       </c>
-      <c r="J19" s="49"/>
-      <c r="K19" s="47"/>
-      <c r="L19" s="47"/>
-      <c r="M19" s="47"/>
-      <c r="N19" s="47"/>
-      <c r="O19" s="47"/>
-      <c r="P19" s="56"/>
-      <c r="Q19" s="56"/>
-      <c r="R19" s="56"/>
-      <c r="S19" s="56"/>
+      <c r="J19" s="48"/>
+      <c r="K19" s="46"/>
+      <c r="L19" s="46"/>
+      <c r="M19" s="46"/>
+      <c r="N19" s="46"/>
+      <c r="O19" s="46"/>
+      <c r="P19" s="55"/>
+      <c r="Q19" s="55"/>
+      <c r="R19" s="55"/>
+      <c r="S19" s="55"/>
       <c r="T19" s="1"/>
-      <c r="V19" s="59"/>
+      <c r="U19" s="58"/>
     </row>
-    <row r="20" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A20" s="23">
         <v>45766</v>
       </c>
       <c r="B20" s="1">
         <v>200</v>
       </c>
-      <c r="C20" s="62">
+      <c r="C20" s="61">
         <v>50</v>
       </c>
       <c r="D20" s="1">
         <v>100</v>
       </c>
-      <c r="E20" s="59"/>
-      <c r="F20" s="61"/>
-      <c r="G20" s="47"/>
-      <c r="H20" s="47"/>
+      <c r="E20" s="58"/>
+      <c r="F20" s="60"/>
+      <c r="G20" s="46"/>
+      <c r="H20" s="46"/>
       <c r="I20" s="23">
         <f t="shared" si="0"/>
         <v>45766</v>
       </c>
-      <c r="J20" s="49">
+      <c r="J20" s="48">
         <v>50</v>
       </c>
-      <c r="K20" s="47"/>
-      <c r="L20" s="47"/>
-      <c r="M20" s="47"/>
-      <c r="N20" s="47"/>
-      <c r="O20" s="47"/>
-      <c r="P20" s="56"/>
-      <c r="Q20" s="56"/>
-      <c r="R20" s="56"/>
-      <c r="S20" s="56"/>
+      <c r="K20" s="46"/>
+      <c r="L20" s="46"/>
+      <c r="M20" s="46"/>
+      <c r="N20" s="46"/>
+      <c r="O20" s="46"/>
+      <c r="P20" s="55"/>
+      <c r="Q20" s="55"/>
+      <c r="R20" s="55"/>
+      <c r="S20" s="55"/>
       <c r="T20" s="1"/>
-      <c r="V20" s="59"/>
+      <c r="U20" s="58"/>
     </row>
-    <row r="21" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A21" s="23">
         <v>45767</v>
       </c>
       <c r="B21" s="1"/>
-      <c r="C21" s="62"/>
-      <c r="D21" s="1"/>
-      <c r="E21" s="59"/>
-      <c r="F21" s="59"/>
-      <c r="G21" s="47"/>
-      <c r="H21" s="47"/>
+      <c r="C21" s="61"/>
+      <c r="D21" s="1">
+        <v>150</v>
+      </c>
+      <c r="E21" s="58"/>
+      <c r="F21" s="58">
+        <v>250</v>
+      </c>
+      <c r="G21" s="46"/>
+      <c r="H21" s="46"/>
       <c r="I21" s="23">
         <f t="shared" si="0"/>
         <v>45767</v>
       </c>
-      <c r="J21" s="49"/>
-      <c r="K21" s="47"/>
-      <c r="L21" s="47"/>
-      <c r="M21" s="47"/>
-      <c r="N21" s="47"/>
-      <c r="O21" s="47"/>
-      <c r="P21" s="56"/>
-      <c r="Q21" s="56"/>
-      <c r="R21" s="56"/>
-      <c r="S21" s="56"/>
+      <c r="J21" s="48"/>
+      <c r="K21" s="46"/>
+      <c r="L21" s="46"/>
+      <c r="M21" s="46"/>
+      <c r="N21" s="46"/>
+      <c r="O21" s="46"/>
+      <c r="P21" s="55">
+        <v>50</v>
+      </c>
+      <c r="Q21" s="55"/>
+      <c r="R21" s="55"/>
+      <c r="S21" s="55"/>
       <c r="T21" s="1"/>
-      <c r="V21" s="59"/>
+      <c r="U21" s="58"/>
     </row>
-    <row r="22" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="23">
         <v>45768</v>
       </c>
       <c r="B22" s="1"/>
-      <c r="C22" s="62"/>
+      <c r="C22" s="61">
+        <v>110</v>
+      </c>
       <c r="D22" s="1"/>
-      <c r="E22" s="59"/>
-      <c r="F22" s="59"/>
-      <c r="G22" s="47"/>
-      <c r="H22" s="47"/>
+      <c r="E22" s="58"/>
+      <c r="F22" s="58">
+        <f>225+15</f>
+        <v>240</v>
+      </c>
+      <c r="G22" s="46">
+        <v>200</v>
+      </c>
+      <c r="H22" s="46"/>
       <c r="I22" s="23">
         <f t="shared" si="0"/>
         <v>45768</v>
       </c>
-      <c r="J22" s="49"/>
-      <c r="K22" s="47"/>
-      <c r="L22" s="47"/>
-      <c r="M22" s="47"/>
-      <c r="N22" s="47"/>
-      <c r="O22" s="47"/>
-      <c r="P22" s="56"/>
-      <c r="Q22" s="56"/>
-      <c r="R22" s="56"/>
-      <c r="S22" s="56"/>
+      <c r="J22" s="48"/>
+      <c r="K22" s="46"/>
+      <c r="L22" s="46"/>
+      <c r="M22" s="46"/>
+      <c r="N22" s="46"/>
+      <c r="O22" s="46"/>
+      <c r="P22" s="55"/>
+      <c r="Q22" s="55"/>
+      <c r="R22" s="55"/>
+      <c r="S22" s="55"/>
       <c r="T22" s="1"/>
-      <c r="V22" s="59"/>
+      <c r="U22" s="58"/>
     </row>
-    <row r="23" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="23">
         <v>45769</v>
       </c>
-      <c r="B23" s="46"/>
-      <c r="C23" s="63"/>
-      <c r="D23" s="45"/>
-      <c r="E23" s="59"/>
-      <c r="F23" s="61"/>
-      <c r="G23" s="48"/>
-      <c r="H23" s="47"/>
+      <c r="B23" s="45"/>
+      <c r="C23" s="62">
+        <v>60</v>
+      </c>
+      <c r="D23" s="44">
+        <v>50</v>
+      </c>
+      <c r="E23" s="58"/>
+      <c r="F23" s="60">
+        <v>50</v>
+      </c>
+      <c r="G23" s="47"/>
+      <c r="H23" s="46"/>
       <c r="I23" s="23">
         <f t="shared" si="0"/>
         <v>45769</v>
       </c>
-      <c r="J23" s="53"/>
-      <c r="K23" s="47"/>
-      <c r="L23" s="47"/>
-      <c r="M23" s="47"/>
-      <c r="N23" s="47"/>
-      <c r="O23" s="47"/>
-      <c r="P23" s="56"/>
-      <c r="Q23" s="56"/>
-      <c r="R23" s="56"/>
-      <c r="S23" s="56"/>
+      <c r="J23" s="52"/>
+      <c r="K23" s="46"/>
+      <c r="L23" s="46"/>
+      <c r="M23" s="46">
+        <v>50</v>
+      </c>
+      <c r="N23" s="46"/>
+      <c r="O23" s="46"/>
+      <c r="P23" s="55"/>
+      <c r="Q23" s="55"/>
+      <c r="R23" s="55">
+        <v>16</v>
+      </c>
+      <c r="S23" s="55"/>
       <c r="T23" s="1"/>
-      <c r="V23" s="59"/>
-      <c r="W23" s="67" t="s">
+      <c r="U23" s="58"/>
+      <c r="V23" s="65" t="s">
         <v>3</v>
       </c>
-      <c r="X23" s="67"/>
-      <c r="Y23" s="67"/>
+      <c r="W23" s="65"/>
+      <c r="X23" s="65"/>
     </row>
-    <row r="24" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A24" s="23">
         <v>45770</v>
       </c>
-      <c r="B24" s="1"/>
-      <c r="C24" s="62"/>
-      <c r="D24" s="1"/>
-      <c r="E24" s="59"/>
-      <c r="F24" s="59"/>
-      <c r="G24" s="47"/>
-      <c r="H24" s="47"/>
+      <c r="B24" s="1">
+        <v>400</v>
+      </c>
+      <c r="C24" s="61">
+        <v>200</v>
+      </c>
+      <c r="D24" s="1">
+        <f>100+200</f>
+        <v>300</v>
+      </c>
+      <c r="E24" s="58">
+        <v>500</v>
+      </c>
+      <c r="F24" s="58">
+        <f>65+150</f>
+        <v>215</v>
+      </c>
+      <c r="G24" s="46">
+        <v>500</v>
+      </c>
+      <c r="H24" s="46">
+        <v>400</v>
+      </c>
       <c r="I24" s="23">
         <f t="shared" si="0"/>
         <v>45770</v>
       </c>
-      <c r="J24" s="49"/>
-      <c r="K24" s="47"/>
-      <c r="L24" s="47"/>
-      <c r="M24" s="47"/>
-      <c r="N24" s="47"/>
-      <c r="O24" s="47"/>
-      <c r="P24" s="56"/>
-      <c r="Q24" s="56"/>
-      <c r="R24" s="56"/>
-      <c r="S24" s="56"/>
-      <c r="T24" s="1"/>
-      <c r="V24" s="59"/>
-      <c r="W24" s="68">
+      <c r="J24" s="48"/>
+      <c r="K24" s="46">
+        <v>200</v>
+      </c>
+      <c r="L24" s="46"/>
+      <c r="M24" s="46">
+        <v>400</v>
+      </c>
+      <c r="N24" s="46">
+        <v>100</v>
+      </c>
+      <c r="O24" s="46"/>
+      <c r="P24" s="55">
+        <v>150</v>
+      </c>
+      <c r="Q24" s="55">
+        <v>150</v>
+      </c>
+      <c r="R24" s="55">
+        <f>100+400+391</f>
+        <v>891</v>
+      </c>
+      <c r="S24" s="55">
+        <v>100</v>
+      </c>
+      <c r="T24" s="1">
+        <v>500</v>
+      </c>
+      <c r="U24" s="58">
+        <v>600</v>
+      </c>
+      <c r="V24" s="66">
         <f>+B37+D37+T37</f>
         <v>0</v>
       </c>
-      <c r="X24" s="68"/>
-      <c r="Y24" s="68"/>
+      <c r="W24" s="66"/>
+      <c r="X24" s="66"/>
     </row>
-    <row r="25" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="A25" s="31">
+    <row r="25" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A25" s="30">
         <v>45771</v>
       </c>
       <c r="B25" s="1"/>
-      <c r="C25" s="62"/>
-      <c r="D25" s="45"/>
-      <c r="E25" s="59"/>
-      <c r="F25" s="61"/>
-      <c r="G25" s="47"/>
-      <c r="H25" s="47"/>
-      <c r="I25" s="31">
+      <c r="C25" s="61"/>
+      <c r="D25" s="44"/>
+      <c r="E25" s="58"/>
+      <c r="F25" s="60"/>
+      <c r="G25" s="46"/>
+      <c r="H25" s="46"/>
+      <c r="I25" s="30">
         <f t="shared" si="0"/>
         <v>45771</v>
       </c>
-      <c r="J25" s="49"/>
-      <c r="K25" s="47"/>
-      <c r="L25" s="47"/>
-      <c r="M25" s="47"/>
-      <c r="N25" s="47"/>
-      <c r="O25" s="47"/>
-      <c r="P25" s="56"/>
-      <c r="Q25" s="56"/>
-      <c r="R25" s="56"/>
-      <c r="S25" s="56"/>
+      <c r="J25" s="48"/>
+      <c r="K25" s="46"/>
+      <c r="L25" s="46"/>
+      <c r="M25" s="46"/>
+      <c r="N25" s="46"/>
+      <c r="O25" s="46"/>
+      <c r="P25" s="55"/>
+      <c r="Q25" s="55"/>
+      <c r="R25" s="55"/>
+      <c r="S25" s="55"/>
       <c r="T25" s="1"/>
-      <c r="V25" s="59"/>
+      <c r="U25" s="58"/>
     </row>
-    <row r="26" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:25" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="23">
         <v>45772</v>
       </c>
-      <c r="B26" s="1"/>
-      <c r="C26" s="62"/>
-      <c r="D26" s="1"/>
-      <c r="E26" s="59"/>
-      <c r="F26" s="59"/>
-      <c r="G26" s="47"/>
-      <c r="H26" s="47"/>
+      <c r="B26" s="1">
+        <v>35</v>
+      </c>
+      <c r="C26" s="61"/>
+      <c r="D26" s="1">
+        <v>100</v>
+      </c>
+      <c r="E26" s="58"/>
+      <c r="F26" s="58">
+        <v>10</v>
+      </c>
+      <c r="G26" s="46"/>
+      <c r="H26" s="46"/>
       <c r="I26" s="23">
         <f t="shared" si="0"/>
         <v>45772</v>
       </c>
-      <c r="J26" s="49"/>
-      <c r="K26" s="47"/>
-      <c r="L26" s="47"/>
-      <c r="M26" s="47"/>
-      <c r="N26" s="47"/>
-      <c r="O26" s="47"/>
-      <c r="P26" s="57"/>
-      <c r="Q26" s="57"/>
-      <c r="R26" s="56"/>
-      <c r="S26" s="56"/>
+      <c r="J26" s="48"/>
+      <c r="K26" s="46"/>
+      <c r="L26" s="46"/>
+      <c r="M26" s="46"/>
+      <c r="N26" s="46"/>
+      <c r="O26" s="46"/>
+      <c r="P26" s="56"/>
+      <c r="Q26" s="56"/>
+      <c r="R26" s="55"/>
+      <c r="S26" s="55"/>
       <c r="T26" s="1"/>
-      <c r="V26" s="59"/>
+      <c r="U26" s="58"/>
     </row>
-    <row r="27" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="23">
         <v>45773</v>
       </c>
       <c r="B27" s="1"/>
-      <c r="C27" s="62"/>
+      <c r="C27" s="61"/>
       <c r="D27" s="1"/>
-      <c r="E27" s="59"/>
-      <c r="F27" s="59"/>
-      <c r="G27" s="47"/>
-      <c r="H27" s="47"/>
+      <c r="E27" s="58"/>
+      <c r="F27" s="58"/>
+      <c r="G27" s="46"/>
+      <c r="H27" s="46"/>
       <c r="I27" s="23">
         <f t="shared" si="0"/>
         <v>45773</v>
       </c>
-      <c r="J27" s="49"/>
-      <c r="K27" s="47"/>
-      <c r="L27" s="51"/>
-      <c r="M27" s="47"/>
-      <c r="N27" s="47"/>
-      <c r="O27" s="47"/>
-      <c r="P27" s="56"/>
-      <c r="Q27" s="56"/>
-      <c r="R27" s="57"/>
-      <c r="S27" s="56"/>
+      <c r="J27" s="48"/>
+      <c r="K27" s="46"/>
+      <c r="L27" s="50"/>
+      <c r="M27" s="46"/>
+      <c r="N27" s="46"/>
+      <c r="O27" s="46"/>
+      <c r="P27" s="55"/>
+      <c r="Q27" s="55"/>
+      <c r="R27" s="56"/>
+      <c r="S27" s="55"/>
       <c r="T27" s="1"/>
-      <c r="V27" s="59"/>
-      <c r="W27" s="7" t="s">
+      <c r="U27" s="58"/>
+      <c r="V27" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="X27" s="6" t="s">
+      <c r="W27" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="Y27" s="8" t="s">
+      <c r="X27" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="Z27" s="18" t="s">
+      <c r="Y27" s="18" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:25" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="23">
         <v>45774</v>
       </c>
       <c r="B28" s="1"/>
-      <c r="C28" s="62"/>
+      <c r="C28" s="61"/>
       <c r="D28" s="1"/>
-      <c r="E28" s="59"/>
-      <c r="F28" s="59"/>
-      <c r="G28" s="47"/>
-      <c r="H28" s="47"/>
+      <c r="E28" s="58"/>
+      <c r="F28" s="58"/>
+      <c r="G28" s="46"/>
+      <c r="H28" s="46"/>
       <c r="I28" s="23">
         <f t="shared" si="0"/>
         <v>45774</v>
       </c>
-      <c r="J28" s="54"/>
-      <c r="K28" s="47"/>
-      <c r="L28" s="47"/>
-      <c r="M28" s="47"/>
-      <c r="N28" s="47"/>
-      <c r="O28" s="47"/>
-      <c r="P28" s="56"/>
-      <c r="Q28" s="58"/>
-      <c r="R28" s="56"/>
-      <c r="S28" s="56"/>
+      <c r="J28" s="53"/>
+      <c r="K28" s="46"/>
+      <c r="L28" s="46"/>
+      <c r="M28" s="46"/>
+      <c r="N28" s="46"/>
+      <c r="O28" s="46"/>
+      <c r="P28" s="55"/>
+      <c r="Q28" s="57"/>
+      <c r="R28" s="55"/>
+      <c r="S28" s="55"/>
       <c r="T28" s="1"/>
-      <c r="V28" s="59"/>
-      <c r="W28" s="4">
+      <c r="U28" s="58"/>
+      <c r="V28" s="4">
         <f>+G37+H37+K37+L37+M37+N37+O37+J37</f>
         <v>0</v>
       </c>
-      <c r="X28" s="4">
+      <c r="W28" s="4">
         <f>P35+P37+Q35+Q37+R37+S35+S37</f>
         <v>0</v>
       </c>
-      <c r="Y28" s="4">
+      <c r="X28" s="4">
         <f>+G35+E35+B35+C35+J35+K35+L35+M35+F35+H35+N35+O35+T35+D35</f>
         <v>38900</v>
       </c>
-      <c r="Z28">
+      <c r="Y28">
         <f>+C15+G8+M14+N25+P20</f>
         <v>650</v>
       </c>
     </row>
-    <row r="29" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="23">
         <v>45775</v>
       </c>
       <c r="B29" s="1"/>
-      <c r="C29" s="62"/>
+      <c r="C29" s="61"/>
       <c r="D29" s="1"/>
-      <c r="E29" s="59"/>
-      <c r="F29" s="59"/>
-      <c r="G29" s="47"/>
-      <c r="H29" s="47"/>
+      <c r="E29" s="58"/>
+      <c r="F29" s="58"/>
+      <c r="G29" s="46"/>
+      <c r="H29" s="46"/>
       <c r="I29" s="23">
         <f t="shared" si="0"/>
         <v>45775</v>
       </c>
-      <c r="J29" s="49"/>
-      <c r="K29" s="47"/>
-      <c r="L29" s="47"/>
-      <c r="M29" s="47"/>
-      <c r="N29" s="47"/>
-      <c r="O29" s="47"/>
-      <c r="P29" s="56"/>
-      <c r="Q29" s="56"/>
-      <c r="R29" s="56"/>
-      <c r="S29" s="56"/>
+      <c r="J29" s="48"/>
+      <c r="K29" s="46"/>
+      <c r="L29" s="46"/>
+      <c r="M29" s="46"/>
+      <c r="N29" s="46"/>
+      <c r="O29" s="46"/>
+      <c r="P29" s="55"/>
+      <c r="Q29" s="55"/>
+      <c r="R29" s="55"/>
+      <c r="S29" s="55"/>
       <c r="T29" s="1"/>
-      <c r="V29" s="59"/>
+      <c r="U29" s="58"/>
     </row>
-    <row r="30" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A30" s="23">
         <v>45776</v>
       </c>
       <c r="B30" s="1"/>
-      <c r="C30" s="63"/>
-      <c r="D30" s="45"/>
-      <c r="E30" s="59"/>
-      <c r="F30" s="61"/>
-      <c r="G30" s="48"/>
-      <c r="H30" s="47"/>
+      <c r="C30" s="62"/>
+      <c r="D30" s="44"/>
+      <c r="E30" s="58"/>
+      <c r="F30" s="60"/>
+      <c r="G30" s="47"/>
+      <c r="H30" s="46"/>
       <c r="I30" s="23">
         <f t="shared" si="0"/>
         <v>45776</v>
       </c>
-      <c r="J30" s="53"/>
-      <c r="K30" s="47"/>
-      <c r="L30" s="47"/>
-      <c r="M30" s="47"/>
-      <c r="N30" s="47"/>
-      <c r="O30" s="47"/>
-      <c r="P30" s="56"/>
-      <c r="Q30" s="56"/>
-      <c r="R30" s="56"/>
-      <c r="S30" s="56"/>
+      <c r="J30" s="52"/>
+      <c r="K30" s="46"/>
+      <c r="L30" s="46"/>
+      <c r="M30" s="46"/>
+      <c r="N30" s="46"/>
+      <c r="O30" s="46"/>
+      <c r="P30" s="55"/>
+      <c r="Q30" s="55"/>
+      <c r="R30" s="55"/>
+      <c r="S30" s="55"/>
       <c r="T30" s="1"/>
-      <c r="V30" s="59"/>
+      <c r="U30" s="58"/>
     </row>
-    <row r="31" spans="1:26" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:25" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="23">
         <v>45777</v>
       </c>
       <c r="B31" s="1"/>
-      <c r="C31" s="62"/>
+      <c r="C31" s="61"/>
       <c r="D31" s="1"/>
-      <c r="E31" s="59"/>
-      <c r="F31" s="59"/>
-      <c r="G31" s="47"/>
-      <c r="H31" s="47"/>
+      <c r="E31" s="58"/>
+      <c r="F31" s="58"/>
+      <c r="G31" s="46"/>
+      <c r="H31" s="46"/>
       <c r="I31" s="23">
         <f t="shared" si="0"/>
         <v>45777</v>
       </c>
-      <c r="J31" s="54"/>
-      <c r="K31" s="55"/>
-      <c r="L31" s="47"/>
-      <c r="M31" s="47"/>
-      <c r="N31" s="47"/>
-      <c r="O31" s="47"/>
-      <c r="P31" s="56"/>
-      <c r="Q31" s="56"/>
-      <c r="R31" s="56"/>
-      <c r="S31" s="56"/>
+      <c r="J31" s="53"/>
+      <c r="K31" s="54"/>
+      <c r="L31" s="46"/>
+      <c r="M31" s="46"/>
+      <c r="N31" s="46"/>
+      <c r="O31" s="46"/>
+      <c r="P31" s="55"/>
+      <c r="Q31" s="55"/>
+      <c r="R31" s="55"/>
+      <c r="S31" s="55"/>
       <c r="T31" s="1"/>
-      <c r="V31" s="59"/>
-      <c r="X31" s="37"/>
-      <c r="Y31" t="s">
-        <v>28</v>
+      <c r="U31" s="58"/>
+      <c r="W31" s="36"/>
+      <c r="X31" t="s">
+        <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:26" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:25" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="23"/>
-      <c r="B32" s="41"/>
-      <c r="E32" s="42"/>
-      <c r="F32" s="43"/>
+      <c r="B32" s="40"/>
+      <c r="E32" s="41"/>
+      <c r="F32" s="42"/>
       <c r="I32" s="23"/>
-      <c r="J32" s="44"/>
-      <c r="L32" s="40"/>
-      <c r="M32" s="43"/>
-      <c r="P32" s="40"/>
-      <c r="Q32" s="40"/>
-      <c r="S32" s="40"/>
-      <c r="X32" s="11"/>
-      <c r="Y32">
+      <c r="J32" s="43"/>
+      <c r="L32" s="39"/>
+      <c r="M32" s="42"/>
+      <c r="P32" s="39"/>
+      <c r="Q32" s="39"/>
+      <c r="S32" s="39"/>
+      <c r="W32" s="11"/>
+      <c r="X32">
         <v>1500</v>
       </c>
     </row>
-    <row r="33" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="23" t="s">
-        <v>9</v>
+    <row r="33" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="67" t="s">
+        <v>10</v>
       </c>
       <c r="B33">
         <f t="shared" ref="B33:E33" si="1">SUM(B2:B32)</f>
-        <v>2591.71</v>
+        <v>3026.71</v>
       </c>
       <c r="C33">
         <f t="shared" si="1"/>
-        <v>3615.71</v>
+        <v>3985.71</v>
       </c>
       <c r="D33">
         <f t="shared" si="1"/>
-        <v>4143.97</v>
+        <v>4743.97</v>
       </c>
       <c r="E33">
         <f t="shared" si="1"/>
-        <v>985.71</v>
+        <v>1485.71</v>
       </c>
       <c r="F33">
         <f>SUM(F2:F32)</f>
-        <v>8064.45</v>
+        <v>8829.4500000000007</v>
       </c>
       <c r="G33">
         <f>SUM(G2:G32)</f>
-        <v>1835.71</v>
+        <v>2535.71</v>
       </c>
       <c r="H33">
         <f>SUM(H2:H32)</f>
-        <v>2885.71</v>
+        <v>3285.71</v>
       </c>
       <c r="I33" s="27"/>
       <c r="J33">
-        <f t="shared" ref="J33:U33" si="2">SUM(J2:J32)</f>
+        <f t="shared" ref="J33:T33" si="2">SUM(J2:J32)</f>
         <v>1085.71</v>
       </c>
       <c r="K33">
         <f t="shared" si="2"/>
-        <v>1500</v>
+        <v>1700</v>
       </c>
       <c r="L33">
         <f t="shared" si="2"/>
@@ -6347,11 +6773,11 @@
       </c>
       <c r="M33">
         <f t="shared" si="2"/>
-        <v>2145.19</v>
+        <v>2595.19</v>
       </c>
       <c r="N33">
         <f t="shared" si="2"/>
-        <v>2500</v>
+        <v>2600</v>
       </c>
       <c r="O33">
         <f t="shared" si="2"/>
@@ -6359,64 +6785,60 @@
       </c>
       <c r="P33">
         <f t="shared" si="2"/>
-        <v>880.71</v>
+        <v>1080.71</v>
       </c>
       <c r="Q33">
         <f t="shared" si="2"/>
-        <v>985.71</v>
+        <v>1135.71</v>
       </c>
       <c r="R33">
         <f t="shared" si="2"/>
-        <v>3489.98</v>
+        <v>4396.9799999999996</v>
       </c>
       <c r="S33">
         <f t="shared" si="2"/>
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="T33">
         <f t="shared" si="2"/>
-        <v>1235.71</v>
+        <v>1735.71</v>
       </c>
       <c r="U33" s="4">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="V33" s="4">
         <f>SUM(الجدول1[[#All],[عمود17]])</f>
-        <v>300</v>
+        <v>900</v>
       </c>
     </row>
-    <row r="34" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="30" t="s">
-        <v>33</v>
+    <row r="34" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="68" t="s">
+        <v>11</v>
       </c>
       <c r="B34" s="26">
         <f>3000-B33</f>
-        <v>408.28999999999996</v>
+        <v>-26.710000000000036</v>
       </c>
       <c r="C34" s="26">
         <f>3000-C33</f>
-        <v>-615.71</v>
+        <v>-985.71</v>
       </c>
       <c r="D34" s="26">
         <f>3000-D33</f>
-        <v>-1143.9700000000003</v>
+        <v>-1743.9700000000003</v>
       </c>
       <c r="E34" s="26">
         <f>3000-E33</f>
-        <v>2014.29</v>
+        <v>1514.29</v>
       </c>
       <c r="F34" s="26">
         <f>4000-F33</f>
-        <v>-4064.45</v>
+        <v>-4829.4500000000007</v>
       </c>
       <c r="G34" s="26">
         <f>3000-G33</f>
-        <v>1164.29</v>
+        <v>464.28999999999996</v>
       </c>
       <c r="H34" s="26">
         <f>3000-H33</f>
-        <v>114.28999999999996</v>
+        <v>-285.71000000000004</v>
       </c>
       <c r="I34" s="27"/>
       <c r="J34">
@@ -6425,7 +6847,7 @@
       </c>
       <c r="K34">
         <f>2000-K33</f>
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="L34">
         <f>3000-L33</f>
@@ -6433,11 +6855,11 @@
       </c>
       <c r="M34">
         <f>2700-M33</f>
-        <v>554.80999999999995</v>
+        <v>104.80999999999995</v>
       </c>
       <c r="N34">
         <f>2700-N33</f>
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="O34">
         <f>1000-O33</f>
@@ -6445,36 +6867,35 @@
       </c>
       <c r="P34">
         <f>1500-P33</f>
-        <v>619.29</v>
+        <v>419.28999999999996</v>
       </c>
       <c r="Q34">
         <f>2000-Q33</f>
-        <v>1014.29</v>
+        <v>864.29</v>
       </c>
       <c r="R34" s="25">
         <f>0-R33</f>
-        <v>-3489.98</v>
+        <v>-4396.9799999999996</v>
       </c>
       <c r="S34">
         <f>400-S33</f>
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="T34">
         <f>3000-T33</f>
-        <v>1764.29</v>
-      </c>
-      <c r="U34" s="4"/>
-      <c r="V34" s="4">
-        <f>2000-V33</f>
-        <v>1700</v>
-      </c>
-      <c r="X34" s="10" t="s">
+        <v>1264.29</v>
+      </c>
+      <c r="U34" s="4">
+        <f>2000-U33</f>
+        <v>1100</v>
+      </c>
+      <c r="W34" s="10" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="35" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="23" t="s">
-        <v>32</v>
+    <row r="35" spans="1:23" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="67" t="s">
+        <v>7</v>
       </c>
       <c r="B35" s="5">
         <v>3000</v>
@@ -6522,24 +6943,24 @@
       <c r="Q35" s="14">
         <v>2000</v>
       </c>
-      <c r="S35" s="34">
+      <c r="S35" s="33">
         <v>500</v>
       </c>
-      <c r="T35" s="38">
+      <c r="T35" s="37">
         <v>3000</v>
       </c>
-      <c r="V35" s="38">
+      <c r="U35" s="37">
         <v>2000</v>
       </c>
-      <c r="W35" s="11"/>
-      <c r="X35">
+      <c r="V35" s="11"/>
+      <c r="W35">
         <f>+C37+E37+F37</f>
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A36" s="23" t="s">
-        <v>7</v>
+    <row r="36" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A36" s="67" t="s">
+        <v>8</v>
       </c>
       <c r="B36" s="9">
         <f>2000-2000</f>
@@ -6588,11 +7009,10 @@
         <v>0</v>
       </c>
       <c r="U36" s="4"/>
-      <c r="V36" s="4"/>
     </row>
-    <row r="37" spans="1:24" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="23" t="s">
-        <v>8</v>
+    <row r="37" spans="1:23" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="67" t="s">
+        <v>9</v>
       </c>
       <c r="B37" s="10">
         <f>0*0.06</f>
@@ -6623,7 +7043,7 @@
         <v>0</v>
       </c>
       <c r="I37" s="27"/>
-      <c r="J37" s="39">
+      <c r="J37" s="38">
         <v>0</v>
       </c>
       <c r="K37" s="3">
@@ -6654,51 +7074,51 @@
         <f>(0/2)-P35-P37-Q35-Q37-S35-S37</f>
         <v>-4000</v>
       </c>
-      <c r="S37" s="60">
+      <c r="S37" s="59">
         <v>0</v>
       </c>
       <c r="T37" s="24">
         <f>0*0.06</f>
         <v>0</v>
       </c>
-      <c r="V37" s="35">
+      <c r="U37" s="34">
         <v>0</v>
       </c>
-      <c r="X37" s="36" t="s">
-        <v>29</v>
+      <c r="W37" s="35" t="s">
+        <v>31</v>
       </c>
     </row>
-    <row r="38" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A38" s="23" t="s">
-        <v>10</v>
+    <row r="38" spans="1:23" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="67" t="s">
+        <v>12</v>
       </c>
       <c r="B38" s="22">
         <f>B34-B36+B37</f>
-        <v>408.28999999999996</v>
+        <v>-26.710000000000036</v>
       </c>
       <c r="C38">
         <f t="shared" ref="C38:H38" si="3">+C34+C37-C36</f>
-        <v>-615.71</v>
+        <v>-985.71</v>
       </c>
       <c r="D38">
         <f>+D34+D37-D36</f>
-        <v>-1143.9700000000003</v>
+        <v>-1743.9700000000003</v>
       </c>
       <c r="E38">
         <f>+E34+E37-E36</f>
-        <v>2014.29</v>
+        <v>1514.29</v>
       </c>
       <c r="F38">
         <f>+F34+F37-F36</f>
-        <v>-4064.45</v>
+        <v>-4829.4500000000007</v>
       </c>
       <c r="G38">
         <f>+G34+G37-G36</f>
-        <v>1164.29</v>
+        <v>464.28999999999996</v>
       </c>
       <c r="H38">
         <f t="shared" si="3"/>
-        <v>114.28999999999996</v>
+        <v>-285.71000000000004</v>
       </c>
       <c r="I38" s="27"/>
       <c r="J38">
@@ -6707,7 +7127,7 @@
       </c>
       <c r="K38">
         <f>+K34+K37-K36</f>
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="L38">
         <f>+L34+L37-L36</f>
@@ -6715,11 +7135,11 @@
       </c>
       <c r="M38">
         <f>+M34+M37-M36</f>
-        <v>554.80999999999995</v>
+        <v>104.80999999999995</v>
       </c>
       <c r="N38">
         <f>N34+N37-N36</f>
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="O38">
         <f>+O34+O37-O36</f>
@@ -6727,72 +7147,67 @@
       </c>
       <c r="P38">
         <f>+P34+P37</f>
-        <v>619.29</v>
+        <v>419.28999999999996</v>
       </c>
       <c r="Q38">
         <f>+Q34+Q37-Q36</f>
-        <v>1014.29</v>
+        <v>864.29</v>
       </c>
       <c r="R38">
         <f>+R34+R37-R36</f>
-        <v>-7489.98</v>
+        <v>-8396.98</v>
       </c>
       <c r="S38">
+        <f>+S34+S37</f>
         <v>0</v>
       </c>
       <c r="T38">
         <f>+T34+T37-T36</f>
-        <v>1764.29</v>
+        <v>1264.29</v>
       </c>
       <c r="U38" s="4"/>
-      <c r="V38" s="4"/>
-      <c r="X38" s="11">
+      <c r="W38" s="11">
         <f>0</f>
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A39" s="13"/>
       <c r="D39" s="22" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
-    <row r="40" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A40" s="13"/>
       <c r="I40"/>
     </row>
-    <row r="41" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A41" s="12"/>
       <c r="F41">
         <f>58015.69-10000</f>
         <v>48015.69</v>
       </c>
     </row>
-    <row r="42" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A42" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="W23:Y23"/>
-    <mergeCell ref="W24:Y24"/>
+    <mergeCell ref="V23:X23"/>
+    <mergeCell ref="V24:X24"/>
   </mergeCells>
   <conditionalFormatting sqref="B34:H34">
-    <cfRule type="cellIs" dxfId="3" priority="4" operator="lessThan">
+    <cfRule type="cellIs" dxfId="2" priority="4" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B38:H38 J38:V38">
-    <cfRule type="cellIs" dxfId="2" priority="7" operator="lessThan">
+  <conditionalFormatting sqref="B38:H38 J38:U38">
+    <cfRule type="cellIs" dxfId="1" priority="7" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J34:Q34 B38:H38 J38:V38">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S34:V34">
-    <cfRule type="cellIs" dxfId="0" priority="3" operator="lessThan">
+  <conditionalFormatting sqref="J34:Q34 S34:U34 B38:H38 J38:U38">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>